<commit_message>
jsonissuefixed.switch to v13. CGA score update preparing.
</commit_message>
<xml_diff>
--- a/2025_demo/GlycoMSP_MAS_v2_template.xlsx
+++ b/2025_demo/GlycoMSP_MAS_v2_template.xlsx
@@ -1,23 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\其他電腦\My Computer\GlycoMSParser\2025_demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5807AD-93F0-43D3-B7E6-62F96B569C63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511F1B22-9344-4959-A3F5-C19330DC4902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{CFD31651-57D7-40EF-BE95-C7417EC3B9A0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{CFD31651-57D7-40EF-BE95-C7417EC3B9A0}"/>
   </bookViews>
   <sheets>
     <sheet name="MSlist" sheetId="6" r:id="rId1"/>
     <sheet name="ionlist" sheetId="4" r:id="rId2"/>
-    <sheet name="some confrimation" sheetId="13" r:id="rId3"/>
-    <sheet name="interpretation" sheetId="14" r:id="rId4"/>
-    <sheet name="readme_pureMAS_and_ion_detail" sheetId="12" r:id="rId5"/>
+    <sheet name="interpretation_v2" sheetId="16" r:id="rId3"/>
+    <sheet name="TargetHierarchy" sheetId="17" r:id="rId4"/>
+    <sheet name="motifpolicy2" sheetId="20" r:id="rId5"/>
+    <sheet name="工作表3" sheetId="19" r:id="rId6"/>
+    <sheet name="MotifPolicy" sheetId="18" r:id="rId7"/>
+    <sheet name="some confrimation" sheetId="13" r:id="rId8"/>
+    <sheet name="interpretation" sheetId="14" r:id="rId9"/>
+    <sheet name="readme_pureMAS_and_ion_detail" sheetId="12" r:id="rId10"/>
+    <sheet name="interpretation (2)" sheetId="15" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">ionlist!$A$1:$K$1</definedName>
@@ -44,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="216">
   <si>
     <t>note</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -417,10 +423,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>BY</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -788,6 +790,732 @@
   </si>
   <si>
     <t>Fragmentation mass</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>target_id</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>target_level</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>parent_target_id</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>target_group</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>ion_struct_id</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>ion_role</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>logic</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>SialylLacNAc</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>motif</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>LacNAc_family</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>Neu5Ac(a2-3)Gal(b1-4)GlcNAc-</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>support</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>AND</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>LeX</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>Lewis_terminal</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>Gal(b1-4)[Fuc(a1-3)]GlcNAc-</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>target_id</t>
+  </si>
+  <si>
+    <t>target_level</t>
+  </si>
+  <si>
+    <t>parent_target_id</t>
+  </si>
+  <si>
+    <t>target_group</t>
+  </si>
+  <si>
+    <t>ion_struct_id</t>
+  </si>
+  <si>
+    <t>ion_role</t>
+  </si>
+  <si>
+    <t>logic</t>
+  </si>
+  <si>
+    <t>min_hits</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>charge_mode_required</t>
+  </si>
+  <si>
+    <t>derivatization_required</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>SialylLacNAc</t>
+  </si>
+  <si>
+    <t>motif</t>
+  </si>
+  <si>
+    <t>LacNAc_family</t>
+  </si>
+  <si>
+    <t>Neu5Ac(a2-3)Gal(b1-4)GlcNAc-</t>
+  </si>
+  <si>
+    <t>support</t>
+  </si>
+  <si>
+    <t>AND</t>
+  </si>
+  <si>
+    <t>any</t>
+  </si>
+  <si>
+    <t>core evidence for sialylated LacNAc</t>
+  </si>
+  <si>
+    <t>Lewis_terminal</t>
+  </si>
+  <si>
+    <t>Gal(b1-4)[Fuc(a1-3)]GlcNAc-</t>
+  </si>
+  <si>
+    <t>Lewis X evidence</t>
+  </si>
+  <si>
+    <t>LeA</t>
+  </si>
+  <si>
+    <t>Gal(b1-3)[Fuc(a1-4)]GlcNAc-</t>
+  </si>
+  <si>
+    <t>Lewis A evidence</t>
+  </si>
+  <si>
+    <t>exclude</t>
+  </si>
+  <si>
+    <t>penalize LeA-marker when claiming LeX</t>
+  </si>
+  <si>
+    <t>penalize LeX-marker when claiming LeA</t>
+  </si>
+  <si>
+    <t>sLeX</t>
+  </si>
+  <si>
+    <t>Neu5Ac(a2-3)Gal(b1-4)[Fuca1-3]GlcNAc-</t>
+  </si>
+  <si>
+    <t>sLeX implies SialylLacNAc context</t>
+  </si>
+  <si>
+    <t>allow partial support if sLeX fragment missing</t>
+  </si>
+  <si>
+    <t>B</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LacNAc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gal(b1-4)GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>580-14</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LacDiNAc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BGH1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fuc(a1-2)Gal(b1-3)GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BGH1_MS3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Oxo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BGH2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BGH2_MS3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fuc(a1-2)Gal(b1-4)GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>638-MeO (C3 elimination)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>α</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-l-Fucp-(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>2)-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>β</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-d-Galp-(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>3)-[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>α</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-l-Fucp-(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>4)]-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>β</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-d-GlcpNAc-(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>3)-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>β</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-d-Galp-(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>4)-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>β</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-d-Glcp</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C3 elimination</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fuc(a1-2)Gal(b1-4)[-dCH3OH]GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[Fuc(a1-4)][-dCH3OH]GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LeB_MS3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LeX_MS3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LeA_MS3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>434-32 (C3 elimination), in paper it is 402.0 but I think should be 402.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LeY_MS3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BZ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fuc(a1-2)Gal(b1-4)-GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sLeX_MS3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Neu5Ac(a2-3)Gal(b1-4)-GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>-[dCH3OH]GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>260-MeO (C3 elimination)  -32.0419 OR 32.0262???</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LacNAc</t>
+  </si>
+  <si>
+    <t>B</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gal(b1-4)GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LacNAc (Type2)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LacNAc (Type1)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gal(b1-3)GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SialylHex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SialylHex-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sugar</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sialyl terminal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>penalize if Neu5Ac is not allowed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>penalize if Neu5Gc is not allowed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ion_struct_id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GalNAc(b1-4)GlcNAc-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>parent_target_id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>child_target_id</t>
+  </si>
+  <si>
+    <t>Type1_chain</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Type2_chain</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gal(b1-3)GlcNAc backbone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gal(b1-4)GlcNAc backbone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>H1</t>
+  </si>
+  <si>
+    <t>H2</t>
+  </si>
+  <si>
+    <t>H2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LeX</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>H type-1 terminal (Fuc a1-2 on Gal)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>H type-2 terminal (Fuc a1-2 on Gal)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lewis A (Fuc a1-4 on GlcNAc)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lewis X (Fuc a1-3 on GlcNAc)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flag_id</t>
+  </si>
+  <si>
+    <t>activation_mode</t>
+  </si>
+  <si>
+    <t>include_descendants</t>
+  </si>
+  <si>
+    <t>weight_multiplier</t>
+  </si>
+  <si>
+    <t>AllowABH</t>
+  </si>
+  <si>
+    <t>enable</t>
+  </si>
+  <si>
+    <t>allow H type-1</t>
+  </si>
+  <si>
+    <t>allow H type-2</t>
+  </si>
+  <si>
+    <t>AllowLewis</t>
+  </si>
+  <si>
+    <t>allow Lewis A</t>
+  </si>
+  <si>
+    <t>allow Lewis X</t>
+  </si>
+  <si>
+    <t>PreferLewis</t>
+  </si>
+  <si>
+    <t>prefer</t>
+  </si>
+  <si>
+    <t>optional grouping node + descendants</t>
+  </si>
+  <si>
+    <t>Fuc(a1-2)Gal(b1-4)GlcNAc-</t>
+  </si>
+  <si>
+    <t>Fuc(a1-2)Gal(b1-3)GlcNAc-</t>
+  </si>
+  <si>
+    <t>BGH1_terminal</t>
+  </si>
+  <si>
+    <t>638 B-ion (H1-type)</t>
+  </si>
+  <si>
+    <t>BGH2_terminal</t>
+  </si>
+  <si>
+    <t>638 B-ion (H2-type)</t>
+  </si>
+  <si>
+    <t>LeA_terminal</t>
+  </si>
+  <si>
+    <t>638 B-ion (LeA-type)</t>
+  </si>
+  <si>
+    <t>LeX_terminal</t>
+  </si>
+  <si>
+    <t>638 B-ion (LeX-type)</t>
+  </si>
+  <si>
+    <t>example</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>motif</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>optional</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>optional?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ion name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ion struct id ref</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Terminal_trisaccharide</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>forbid</t>
+  </si>
+  <si>
+    <t>AllowBGH1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AllowBGH2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AllowLewisA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AllowLewisX</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PreferLewisA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PreferLewisX</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ForbidLewisA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ForbidLewisX</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -795,7 +1523,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -846,6 +1574,21 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="6"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -869,7 +1612,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -882,11 +1625,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1266,7 +2032,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6820557B-6CE2-4FD8-86A4-E2CD52A6D2FD}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="2" width="18.375" customWidth="1"/>
     <col min="3" max="3" width="11.125" customWidth="1"/>
@@ -1598,19 +2364,19 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" t="s">
         <v>45</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>46</v>
-      </c>
-      <c r="C19" t="s">
-        <v>47</v>
       </c>
       <c r="E19">
         <v>2</v>
       </c>
       <c r="G19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1624,15 +2390,106 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7792179-2CDA-4B5E-99B0-403A61C061FC}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE432269-C452-9446-B586-38925AC56B75}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="12.75" customWidth="1"/>
+    <col min="2" max="2" width="20.375" customWidth="1"/>
+    <col min="3" max="3" width="18.375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="18.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="7"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D125B437-E159-4E97-8559-08AC52B2F723}">
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="22.5" customWidth="1"/>
+    <col min="1" max="1" width="22.375" customWidth="1"/>
     <col min="3" max="3" width="23.125" customWidth="1"/>
-    <col min="4" max="4" width="34.5" customWidth="1"/>
-    <col min="5" max="5" width="12.5" customWidth="1"/>
+    <col min="4" max="4" width="34.375" customWidth="1"/>
+    <col min="5" max="5" width="12.375" customWidth="1"/>
     <col min="6" max="6" width="9.125" customWidth="1"/>
     <col min="7" max="7" width="58.375" customWidth="1"/>
     <col min="8" max="8" width="51.125" customWidth="1"/>
@@ -1647,7 +2504,7 @@
         <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D1" t="s">
         <v>15</v>
@@ -1667,7 +2524,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>125</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -1676,7 +2533,7 @@
         <v>638.33820000000003</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>126</v>
       </c>
       <c r="E2" t="s">
         <v>34</v>
@@ -1684,28 +2541,19 @@
       <c r="F2" t="s">
         <v>36</v>
       </c>
-      <c r="G2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>127</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3">
-        <v>656.34879999999998</v>
-      </c>
-      <c r="D3" t="s">
-        <v>32</v>
+        <v>128</v>
+      </c>
+      <c r="C3" s="1">
+        <v>228.12299999999999</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>146</v>
       </c>
       <c r="E3" t="s">
         <v>34</v>
@@ -1713,19 +2561,22 @@
       <c r="F3" t="s">
         <v>36</v>
       </c>
+      <c r="G3" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>129</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4">
-        <v>260.14920000000001</v>
+        <v>638.33820000000003</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>131</v>
       </c>
       <c r="E4" t="s">
         <v>34</v>
@@ -1736,16 +2587,16 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>130</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5">
-        <v>344.17039999999997</v>
+        <v>128</v>
+      </c>
+      <c r="C5" s="1">
+        <v>606.31200000000001</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>135</v>
       </c>
       <c r="E5" t="s">
         <v>34</v>
@@ -1753,19 +2604,22 @@
       <c r="F5" t="s">
         <v>36</v>
       </c>
+      <c r="G5" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
       </c>
       <c r="C6">
-        <v>374.18099999999998</v>
+        <v>260.14920000000001</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="E6" t="s">
         <v>34</v>
@@ -1776,16 +2630,16 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>120</v>
       </c>
       <c r="C7">
-        <v>376.19659999999999</v>
+        <v>505.2756</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>161</v>
       </c>
       <c r="E7" t="s">
         <v>34</v>
@@ -1796,16 +2650,16 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>120</v>
       </c>
       <c r="C8">
-        <v>406.2072</v>
+        <v>464.24900000000002</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>122</v>
       </c>
       <c r="E8" t="s">
         <v>34</v>
@@ -1816,16 +2670,16 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>152</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9">
-        <v>566.28070000000002</v>
+        <v>149</v>
+      </c>
+      <c r="C9" s="1">
+        <v>464.24900000000002</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>153</v>
       </c>
       <c r="E9" t="s">
         <v>34</v>
@@ -1836,16 +2690,16 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>151</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>149</v>
       </c>
       <c r="C10">
-        <v>580.29639999999995</v>
+        <v>464.24900000000002</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>150</v>
       </c>
       <c r="E10" t="s">
         <v>34</v>
@@ -1856,16 +2710,16 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C11">
-        <v>999.51189999999997</v>
+        <v>638.33820000000003</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
         <v>34</v>
@@ -1873,22 +2727,19 @@
       <c r="F11" t="s">
         <v>36</v>
       </c>
-      <c r="H11" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="C12">
-        <v>825.42269999999996</v>
+        <v>656.34879999999998</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
         <v>34</v>
@@ -1899,16 +2750,16 @@
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>139</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13">
-        <v>638.33820000000003</v>
-      </c>
-      <c r="D13" t="s">
-        <v>55</v>
+        <v>128</v>
+      </c>
+      <c r="C13" s="1">
+        <v>402.21230000000003</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>136</v>
       </c>
       <c r="E13" t="s">
         <v>34</v>
@@ -1916,19 +2767,22 @@
       <c r="F13" t="s">
         <v>36</v>
       </c>
+      <c r="G13" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="C14">
-        <v>656.34879999999998</v>
+        <v>812.42740000000003</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="E14" t="s">
         <v>34</v>
@@ -1936,19 +2790,22 @@
       <c r="F14" t="s">
         <v>36</v>
       </c>
+      <c r="H14" s="2" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>137</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15">
-        <v>812.42740000000003</v>
+        <v>128</v>
+      </c>
+      <c r="C15" s="1">
+        <v>402.21230000000003</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
+        <v>136</v>
       </c>
       <c r="E15" t="s">
         <v>34</v>
@@ -1956,19 +2813,22 @@
       <c r="F15" t="s">
         <v>36</v>
       </c>
+      <c r="G15" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C16">
-        <v>812.42740000000003</v>
+        <v>638.33820000000003</v>
       </c>
       <c r="D16" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="E16" t="s">
         <v>34</v>
@@ -1976,22 +2836,1264 @@
       <c r="F16" t="s">
         <v>36</v>
       </c>
+      <c r="G16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H16" t="s">
+        <v>27</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17">
+        <v>656.34879999999998</v>
+      </c>
+      <c r="D17" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B18" t="s">
+        <v>128</v>
+      </c>
+      <c r="C18" s="1">
+        <v>432.22280000000001</v>
+      </c>
+      <c r="D18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19">
+        <v>812.42740000000003</v>
+      </c>
+      <c r="D19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>141</v>
+      </c>
+      <c r="B20" t="s">
+        <v>142</v>
+      </c>
+      <c r="C20" s="1">
+        <v>606.31200000000001</v>
+      </c>
+      <c r="D20" t="s">
+        <v>143</v>
+      </c>
+      <c r="E20" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21">
+        <v>344.17039999999997</v>
+      </c>
+      <c r="D21" t="s">
+        <v>51</v>
+      </c>
+      <c r="E21" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22">
+        <v>376.19659999999999</v>
+      </c>
+      <c r="D22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23">
+        <v>374.18099999999998</v>
+      </c>
+      <c r="D23" t="s">
+        <v>52</v>
+      </c>
+      <c r="E23" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24">
+        <v>406.2072</v>
+      </c>
+      <c r="D24" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
+        <v>154</v>
+      </c>
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25">
+        <v>580.29639999999995</v>
+      </c>
+      <c r="D25" t="s">
+        <v>41</v>
+      </c>
+      <c r="E25" t="s">
+        <v>34</v>
+      </c>
+      <c r="F25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
+        <v>155</v>
+      </c>
+      <c r="B26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26">
+        <v>566.28070000000002</v>
+      </c>
+      <c r="D26" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" t="s">
+        <v>34</v>
+      </c>
+      <c r="F26" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27">
+        <v>825.42269999999996</v>
+      </c>
+      <c r="D27" t="s">
+        <v>50</v>
+      </c>
+      <c r="E27" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28">
+        <v>999.51189999999997</v>
+      </c>
+      <c r="D28" t="s">
+        <v>31</v>
+      </c>
+      <c r="E28" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H28" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" t="s">
+        <v>142</v>
+      </c>
+      <c r="C29">
+        <v>793.6</v>
+      </c>
+      <c r="D29" t="s">
+        <v>145</v>
+      </c>
+      <c r="E29" t="s">
+        <v>34</v>
+      </c>
+      <c r="F29" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{D125B437-E159-4E97-8559-08AC52B2F723}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K283">
-      <sortCondition ref="C1"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I29">
+      <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="C28:C29">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F1ABE24-5C3E-4DE8-8A19-1E2068143774}">
+  <dimension ref="A1:M12"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="21.375" customWidth="1"/>
+    <col min="2" max="2" width="20.625" customWidth="1"/>
+    <col min="3" max="3" width="19.75" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="6" width="26.5" customWidth="1"/>
+    <col min="11" max="11" width="17.125" customWidth="1"/>
+    <col min="12" max="12" width="20.25" customWidth="1"/>
+    <col min="13" max="13" width="33.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="33">
+      <c r="A1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I3" s="5">
+        <v>1</v>
+      </c>
+      <c r="J3" s="5">
+        <v>1</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="5">
+        <v>1</v>
+      </c>
+      <c r="J4" s="5">
+        <v>1</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I5" s="5">
+        <v>1</v>
+      </c>
+      <c r="J5" s="5">
+        <v>1</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I6" s="5">
+        <v>1</v>
+      </c>
+      <c r="J6" s="5">
+        <v>1</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I7" s="5">
+        <v>1</v>
+      </c>
+      <c r="J7" s="5">
+        <v>1</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="33">
+      <c r="A8" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I8" s="5">
+        <v>1</v>
+      </c>
+      <c r="J8" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="33">
+      <c r="A9" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I9" s="5">
+        <v>1</v>
+      </c>
+      <c r="J9" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I10" s="5">
+        <v>1</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I11" s="5">
+        <v>1</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" s="7"/>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABF9D4FB-A849-439C-802C-83D42FDCE3EA}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="18.125" customWidth="1"/>
+    <col min="2" max="2" width="27" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>165</v>
+      </c>
+      <c r="B7" t="s">
+        <v>171</v>
+      </c>
+      <c r="C7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>206</v>
+      </c>
+      <c r="B9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>206</v>
+      </c>
+      <c r="B10" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>206</v>
+      </c>
+      <c r="B11" t="s">
+        <v>198</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC41B5F3-E05E-4A4A-8E90-F419DB4B142E}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="23.125" customWidth="1"/>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="3" max="3" width="17.625" customWidth="1"/>
+    <col min="4" max="4" width="16.125" customWidth="1"/>
+    <col min="5" max="5" width="21.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="49.5">
+      <c r="A1" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D4" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D7" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="D8" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10F43228-43AF-4841-8E89-90B9A88581D5}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="33">
+      <c r="A1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="66">
+      <c r="A2" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="66">
+      <c r="A3" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="66">
+      <c r="A4" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="66">
+      <c r="A5" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1BD2AD-7B7D-4DE6-9D29-0FFEA06D7A5B}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="49.5">
+      <c r="A1" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="33">
+      <c r="A2" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="33">
+      <c r="A3" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>1</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="33">
+      <c r="A4" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D4" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>1</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="33">
+      <c r="A5" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="82.5">
+      <c r="A6" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A487D3B1-73FC-471F-BF7D-464BEF914EFC}">
   <dimension ref="D3:F5"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5"/>
   <cols>
     <col min="4" max="4" width="20.375" customWidth="1"/>
     <col min="5" max="5" width="49.25" customWidth="1"/>
@@ -1999,23 +4101,23 @@
   <sheetData>
     <row r="3" spans="4:6">
       <c r="E3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" t="s">
         <v>60</v>
-      </c>
-      <c r="F3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="4" spans="4:6">
       <c r="E4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="4:6">
       <c r="D5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2025,10 +4127,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3EC3B83-AAB3-4F0F-A3D2-3A872002D8E9}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="10.625" customWidth="1"/>
     <col min="2" max="2" width="20.375" customWidth="1"/>
@@ -2036,15 +4138,15 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" t="s">
         <v>66</v>
-      </c>
-      <c r="B3" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2052,7 +4154,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4">
         <v>376.19659999999999</v>
@@ -2060,7 +4162,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
@@ -2071,7 +4173,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
         <v>24</v>
@@ -2086,34 +4188,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7792179-2CDA-4B5E-99B0-403A61C061FC}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="f82b70a8-9591-478e-a6d5-bf315b83c485" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="ドキュメント" ma:contentTypeID="0x010100B01D25D17823C344A9D69518AF56DC62" ma:contentTypeVersion="6" ma:contentTypeDescription="新しいドキュメントを作成します。" ma:contentTypeScope="" ma:versionID="f29605d1c82d3d43c74cd3efc573dd15">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="f82b70a8-9591-478e-a6d5-bf315b83c485" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d7d0483a01e3419b531383906934819f" ns3:_="">
     <xsd:import namespace="f82b70a8-9591-478e-a6d5-bf315b83c485"/>
@@ -2269,10 +4344,37 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="f82b70a8-9591-478e-a6d5-bf315b83c485" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F80E8E46-C8F1-4EA0-9D75-58D6A3F6209E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3840DE93-E5DB-49F7-A595-E7AEB960EE63}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f82b70a8-9591-478e-a6d5-bf315b83c485"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2294,19 +4396,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3840DE93-E5DB-49F7-A595-E7AEB960EE63}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F80E8E46-C8F1-4EA0-9D75-58D6A3F6209E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f82b70a8-9591-478e-a6d5-bf315b83c485"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>